<commit_message>
update pred to w24 of sarima
</commit_message>
<xml_diff>
--- a/dashboard/data_pred.xlsx
+++ b/dashboard/data_pred.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3d9ca122eaf7d8bd/Documents/GitHub/swaper/dashboard/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\swaper\dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{3AD31089-26B7-4772-8C76-D4E1FB2E3CF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{34F9EF85-E417-4C3C-BD4B-54DEAB787BDC}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63494546-645D-40B2-8710-5E72ADE3616C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E3B4F240-1C7B-4534-B2F2-ADBAE75C1F39}"/>
   </bookViews>
@@ -130,10 +130,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -665,6 +661,9 @@
       <c r="C14" s="1">
         <v>609</v>
       </c>
+      <c r="D14">
+        <v>440</v>
+      </c>
       <c r="E14" s="3"/>
     </row>
     <row r="15" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -677,6 +676,9 @@
       <c r="C15" s="1">
         <v>529</v>
       </c>
+      <c r="D15">
+        <v>417</v>
+      </c>
       <c r="E15" s="3"/>
     </row>
     <row r="16" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -689,6 +691,9 @@
       <c r="C16" s="1">
         <v>599</v>
       </c>
+      <c r="D16">
+        <v>425</v>
+      </c>
       <c r="E16" s="3"/>
     </row>
     <row r="17" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -701,6 +706,9 @@
       <c r="C17" s="1">
         <v>569</v>
       </c>
+      <c r="D17">
+        <v>420</v>
+      </c>
       <c r="E17" s="3"/>
     </row>
     <row r="18" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -713,6 +721,9 @@
       <c r="C18" s="1">
         <v>408</v>
       </c>
+      <c r="D18">
+        <v>456</v>
+      </c>
       <c r="E18" s="3"/>
     </row>
     <row r="19" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -725,6 +736,9 @@
       <c r="C19" s="1">
         <v>567</v>
       </c>
+      <c r="D19">
+        <v>319</v>
+      </c>
       <c r="E19" s="3"/>
     </row>
     <row r="20" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -737,6 +751,9 @@
       <c r="C20" s="1">
         <v>573</v>
       </c>
+      <c r="D20">
+        <v>446</v>
+      </c>
       <c r="E20" s="3"/>
     </row>
     <row r="21" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -749,6 +766,9 @@
       <c r="C21" s="1">
         <v>565</v>
       </c>
+      <c r="D21">
+        <v>476</v>
+      </c>
       <c r="E21" s="3"/>
     </row>
     <row r="22" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -761,6 +781,9 @@
       <c r="C22" s="1">
         <v>525</v>
       </c>
+      <c r="D22">
+        <v>460</v>
+      </c>
       <c r="E22" s="3"/>
     </row>
     <row r="23" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -773,6 +796,9 @@
       <c r="C23" s="1">
         <v>688</v>
       </c>
+      <c r="D23">
+        <v>459</v>
+      </c>
       <c r="E23" s="3"/>
     </row>
     <row r="24" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -785,6 +811,9 @@
       <c r="C24" s="1">
         <v>864</v>
       </c>
+      <c r="D24">
+        <v>544</v>
+      </c>
       <c r="E24" s="3"/>
     </row>
     <row r="25" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -796,6 +825,9 @@
       </c>
       <c r="C25" s="1">
         <v>1071</v>
+      </c>
+      <c r="D25">
+        <v>524</v>
       </c>
       <c r="E25" s="3"/>
     </row>

</xml_diff>